<commit_message>
Add Attendance and add logout feature and edit feature and download CSV after changes
</commit_message>
<xml_diff>
--- a/Employees Email id.xlsx
+++ b/Employees Email id.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="112">
   <si>
     <t>Mayur Kumar</t>
   </si>
@@ -107,9 +107,6 @@
     <t>Pratima</t>
   </si>
   <si>
-    <t>Jai Chand</t>
-  </si>
-  <si>
     <t>Anshul Kumar</t>
   </si>
   <si>
@@ -351,6 +348,27 @@
   </si>
   <si>
     <t>Yashpal Thakur</t>
+  </si>
+  <si>
+    <t>Jaichand</t>
+  </si>
+  <si>
+    <t>Rahul Singh</t>
+  </si>
+  <si>
+    <t>Amanjot </t>
+  </si>
+  <si>
+    <t>Nikhil Saini</t>
+  </si>
+  <si>
+    <t>rahul.singh@caglobal.com</t>
+  </si>
+  <si>
+    <t>nikhil.saini@caglobal.com</t>
+  </si>
+  <si>
+    <t>amanjot.singh@caglobal.com</t>
   </si>
 </sst>
 </file>
@@ -429,7 +447,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -438,6 +456,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -775,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="27.796875" style="1" customWidth="1"/>
@@ -784,10 +805,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>101</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -795,7 +816,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -806,7 +827,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -817,7 +838,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4">
         <v>2</v>
@@ -828,7 +849,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -839,7 +860,7 @@
         <v>3</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -850,7 +871,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C7">
         <v>2</v>
@@ -861,7 +882,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8">
         <v>2</v>
@@ -872,7 +893,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -883,7 +904,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -894,7 +915,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -905,7 +926,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -916,7 +937,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C13">
         <v>2</v>
@@ -927,7 +948,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C14">
         <v>2</v>
@@ -938,7 +959,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -946,10 +967,10 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C16">
         <v>2</v>
@@ -960,7 +981,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C17">
         <v>2</v>
@@ -971,7 +992,7 @@
         <v>16</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -982,7 +1003,7 @@
         <v>17</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C19">
         <v>2</v>
@@ -993,7 +1014,7 @@
         <v>18</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C20">
         <v>2</v>
@@ -1004,7 +1025,7 @@
         <v>12</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C21">
         <v>2</v>
@@ -1015,7 +1036,7 @@
         <v>19</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C22">
         <v>2</v>
@@ -1026,7 +1047,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C23">
         <v>2</v>
@@ -1037,7 +1058,7 @@
         <v>21</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C24">
         <v>2</v>
@@ -1048,7 +1069,7 @@
         <v>22</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C25">
         <v>2</v>
@@ -1059,7 +1080,7 @@
         <v>23</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C26">
         <v>2</v>
@@ -1067,10 +1088,10 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="2" t="s">
-        <v>24</v>
+        <v>105</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C27">
         <v>2</v>
@@ -1078,10 +1099,10 @@
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C28">
         <v>2</v>
@@ -1089,10 +1110,10 @@
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C29">
         <v>2</v>
@@ -1100,10 +1121,10 @@
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C30">
         <v>2</v>
@@ -1111,10 +1132,10 @@
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C31">
         <v>2</v>
@@ -1122,10 +1143,10 @@
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C32">
         <v>2</v>
@@ -1133,10 +1154,10 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C33">
         <v>2</v>
@@ -1144,10 +1165,10 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C34">
         <v>2</v>
@@ -1155,10 +1176,10 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C35">
         <v>2</v>
@@ -1166,10 +1187,10 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -1177,10 +1198,10 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C37">
         <v>2</v>
@@ -1188,10 +1209,10 @@
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C38">
         <v>2</v>
@@ -1199,10 +1220,10 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C39">
         <v>2</v>
@@ -1210,10 +1231,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C40">
         <v>2</v>
@@ -1221,10 +1242,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C41">
         <v>2</v>
@@ -1232,10 +1253,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C42">
         <v>2</v>
@@ -1243,10 +1264,10 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C43">
         <v>2</v>
@@ -1254,10 +1275,10 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B44" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>82</v>
       </c>
       <c r="C44">
         <v>2</v>
@@ -1265,10 +1286,10 @@
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B45" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>84</v>
       </c>
       <c r="C45">
         <v>2</v>
@@ -1276,10 +1297,10 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C46">
         <v>2</v>
@@ -1287,10 +1308,10 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C47">
         <v>2</v>
@@ -1298,10 +1319,10 @@
     </row>
     <row r="48" spans="1:3">
       <c r="A48" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C48">
         <v>2</v>
@@ -1309,10 +1330,10 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C49">
         <v>2</v>
@@ -1320,10 +1341,10 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C50">
         <v>2</v>
@@ -1331,10 +1352,10 @@
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C51">
         <v>2</v>
@@ -1342,10 +1363,10 @@
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C52">
         <v>2</v>
@@ -1353,13 +1374,37 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C53">
         <v>2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3">
+      <c r="A54" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3">
+      <c r="A55" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3">
+      <c r="A56" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -1409,6 +1454,9 @@
     <hyperlink ref="B43" r:id="rId42"/>
     <hyperlink ref="B44" r:id="rId43"/>
     <hyperlink ref="B45" r:id="rId44"/>
+    <hyperlink ref="B54" r:id="rId45"/>
+    <hyperlink ref="B55" r:id="rId46"/>
+    <hyperlink ref="B56" r:id="rId47"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>